<commit_message>
Implement cell triangle drawing in UI.
</commit_message>
<xml_diff>
--- a/src/Sudoku.Graphics.UI/Assets/Unused/Icons.xlsx
+++ b/src/Sudoku.Graphics.UI/Assets/Unused/Icons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\source\repos\Sudoku.Graphics\src\Sudoku.Graphics.UI\Assets\Unused\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6C6AC6-3214-4B99-96C1-96CEA70790BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF40B13-4F5C-44B8-9D3D-7F8409C0B779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{298DA60D-454B-478D-B88C-D8BE946E1239}"/>
   </bookViews>
@@ -2024,6 +2024,157 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>457198</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>153025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>432525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>61686</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="12" name="组合 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1537F2EE-F02E-867E-60E2-E6FC03F5E12A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="5613398" y="4097282"/>
+          <a:ext cx="1956527" cy="1686661"/>
+          <a:chOff x="370113" y="871482"/>
+          <a:chExt cx="1956527" cy="1686661"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="等腰三角形 7">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{647846D4-DB6C-5560-FEEA-DF81FE940CE8}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="370113" y="871482"/>
+            <a:ext cx="1956527" cy="1686661"/>
+          </a:xfrm>
+          <a:prstGeom prst="triangle">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="箭头: 环形 10">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B064810-AB24-28A7-2C1A-10DADB50E207}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="2147707">
+            <a:off x="1632857" y="888999"/>
+            <a:ext cx="464458" cy="464458"/>
+          </a:xfrm>
+          <a:prstGeom prst="circularArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="val 7895"/>
+              <a:gd name="adj2" fmla="val 1281339"/>
+              <a:gd name="adj3" fmla="val 20107237"/>
+              <a:gd name="adj4" fmla="val 10800000"/>
+              <a:gd name="adj5" fmla="val 12500"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg2"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
Implement line segment drawing in both API and UI.
</commit_message>
<xml_diff>
--- a/src/Sudoku.Graphics.UI/Assets/Unused/Icons.xlsx
+++ b/src/Sudoku.Graphics.UI/Assets/Unused/Icons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\source\repos\Sudoku.Graphics\src\Sudoku.Graphics.UI\Assets\Unused\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0012B8ED-EBD6-447E-B4A0-FD4986D366FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61E887F-8971-49F3-8FCB-B91BBF3CDCD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{298DA60D-454B-478D-B88C-D8BE946E1239}"/>
   </bookViews>
@@ -5294,6 +5294,61 @@
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>283029</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>10885</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>47172</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>10885</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="89" name="直接连接符 88">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31DBE6C6-5773-4310-A43E-322731238ED3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7420429" y="10889342"/>
+          <a:ext cx="1745343" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="76200">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>